<commit_message>
Agregar lista de compras familiar (5 personas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pZgC66T2WsoYJHMycoAbf
</commit_message>
<xml_diff>
--- a/docs/seguimiento-dieta.xlsx
+++ b/docs/seguimiento-dieta.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menú" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras familia" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menú" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -93,6 +94,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2282,6 +2284,1229 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Estimado (S/)</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Real (S/)</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>Diferencia (S/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pollo (1 kg pechuga + 2 kg pierna/muslo + extra)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4 kg</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="8">
+        <f>IF(E2="","",E2-D2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pescado fresco (jurel/caballa/bonito)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2,5 kg</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3" s="11" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="8">
+        <f>IF(E3="","",E3-D3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Atún en agua</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>6 latas</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="8">
+        <f>IF(E4="","",E4-D4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Carne de res (bistec o molida magra)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="8">
+        <f>IF(E5="","",E5-D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Huevos</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>6 docenas</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="8">
+        <f>IF(E6="","",E6-D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Queso fresco</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>750 g</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="8">
+        <f>IF(E7="","",E7-D7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Yogur natural sin azúcar</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3 kg</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="8">
+        <f>IF(E8="","",E8-D8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Proteínas y lácteos</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Leche (UHT o fresca)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8 L</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="8">
+        <f>IF(E9="","",E9-D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Lentejas</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="8">
+        <f>IF(E10="","",E10-D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Frejoles</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="8">
+        <f>IF(E11="","",E11-D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Quinua</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>750 g</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="8">
+        <f>IF(E12="","",E12-D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Arroz integral</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1,5 kg</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="8">
+        <f>IF(E13="","",E13-D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Arroz blanco</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2 kg</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="8">
+        <f>IF(E14="","",E14-D14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Avena en hojuelas</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1,2 kg</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="8">
+        <f>IF(E15="","",E15-D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pan integral</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>3 bolsas</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="8">
+        <f>IF(E16="","",E16-D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Menestras y granos</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Fideos / pasta</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="8">
+        <f>IF(E17="","",E17-D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Camote</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>3 kg</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="8">
+        <f>IF(E18="","",E18-D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4 kg</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="8">
+        <f>IF(E19="","",E19-D19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tomate</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>3 kg</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="8">
+        <f>IF(E20="","",E20-D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cebolla roja</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>3 kg</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="8">
+        <f>IF(E21="","",E21-D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Zanahoria</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2,5 kg</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="8">
+        <f>IF(E22="","",E22-D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Espinaca</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5 atados</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="8">
+        <f>IF(E23="","",E23-D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Brócoli</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>3 unidades</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="8">
+        <f>IF(E24="","",E24-D24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Zapallo</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1,5 kg</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="8">
+        <f>IF(E25="","",E25-D25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Choclo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>4 unidades</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="8">
+        <f>IF(E26="","",E26-D26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Lechuga</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="8">
+        <f>IF(E27="","",E27-D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Pepino</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="8">
+        <f>IF(E28="","",E28-D28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Arvejas</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>750 g</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="8">
+        <f>IF(E29="","",E29-D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Limones</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1,5 kg</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="8">
+        <f>IF(E30="","",E30-D30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Palta</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>8 unidades</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="8">
+        <f>IF(E31="","",E31-D31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Verduras y tubérculos</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Ajo, culantro, perejil, ají amarillo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>varios</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="8">
+        <f>IF(E32="","",E32-D32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Fruta</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Plátano de seda</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>≈30</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="8">
+        <f>IF(E33="","",E33-D33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Fruta</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Manzana</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>4 kg</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="8">
+        <f>IF(E34="","",E34-D34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Fruta</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Papaya</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>3 medianas</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="8">
+        <f>IF(E35="","",E35-D35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Fruta</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Mandarina</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>3 kg</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="8">
+        <f>IF(E36="","",E36-D36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Fruta</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Naranja</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>3 kg</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="8">
+        <f>IF(E37="","",E37-D37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Fruta</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Fruta de temporada (uvas, fresas, piña)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2 kg</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="8">
+        <f>IF(E38="","",E38-D38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Grasas y frutos secos</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Aceite de oliva extra virgen</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="8">
+        <f>IF(E39="","",E39-D39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Grasas y frutos secos</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Aceite vegetal</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1 L</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="8">
+        <f>IF(E40="","",E40-D40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Grasas y frutos secos</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Maní tostado sin sal</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>600 g</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="8">
+        <f>IF(E41="","",E41-D41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Grasas y frutos secos</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Mantequilla de maní natural</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1 frasco</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E42" s="11" t="n"/>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="8">
+        <f>IF(E42="","",E42-D42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Despensa y antojos controlados</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Condimentos (sal, comino, orégano, ají panca)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>varios</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="8">
+        <f>IF(E43="","",E43-D43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Despensa y antojos controlados</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Azúcar</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E44" s="11" t="n"/>
+      <c r="F44" s="5" t="n"/>
+      <c r="G44" s="8">
+        <f>IF(E44="","",E44-D44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Despensa y antojos controlados</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Antojos: galletas integrales, chocolate amargo, canchita</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>presupuesto</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E45" s="11" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="8">
+        <f>IF(E45="","",E45-D45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D46" s="8">
+        <f>SUM(D2:D45)</f>
+        <v/>
+      </c>
+      <c r="E46" s="8">
+        <f>SUM(E2:E45)</f>
+        <v/>
+      </c>
+      <c r="G46" s="8">
+        <f>IF(E46=0,"",E46-D46)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Agregar porciones por persona y horarios de comida
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pZgC66T2WsoYJHMycoAbf
</commit_message>
<xml_diff>
--- a/docs/seguimiento-dieta.xlsx
+++ b/docs/seguimiento-dieta.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras familia" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menú" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Porciones" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horarios" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -75,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +97,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3729,4 +3737,1024 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Ella</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Él</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>Hijo 18</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Hijo 16</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>Hijo 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Almuerzo: Pollo al horno + quinua + ensalada</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>pollo 150 g, quinua ½ taza</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>pollo 170 g, quinua ½ taza</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>pollo 250 g, quinua 2 taza</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>pollo 200 g, quinua 1½ taza</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>pollo 150 g, quinua 1 taza</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Cena: Lentejas guisadas + huevo + ensalada</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>lentejas ¾ taza, huevo 1</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1 taza, huevo 1</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1½ taza, huevo 2</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1¼ taza, huevo 2</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1 taza, huevo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Almuerzo: Pescado al horno + camote + ensalada</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>pescado 150 g, camote 100 g</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>pescado 170 g, camote 100 g</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>pescado 250 g, camote 350 g</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>pescado 200 g, camote 250 g</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>pescado 150 g, camote 200 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Cena: Sopa de verduras con pollo</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>1 plato, pollo 100 g</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>1 plato, pollo 100 g</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>2 plato, pollo 150 g</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>1½ plato, pollo 120 g</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>1½ plato, pollo 100 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Almuerzo: Estofado de pollo + arroz integral</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>pollo 150 g, arroz ½ taza</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>pollo 170 g, arroz ½ taza</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>pollo 250 g, arroz 2 taza</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>pollo 200 g, arroz 1½ taza</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>pollo 150 g, arroz 1 taza</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Cena: Tortilla de espinaca + camote + ensalada</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>2 huevos, camote 100 g</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>2 huevos, camote 100 g</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>4 huevos, camote 350 g</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>3 huevos, camote 250 g</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>2 huevos, camote 200 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Almuerzo: Ensalada de quinua con atún y ¼ palta</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>atún 1 lata(s), quinua ½ taza</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>atún 1 lata(s), quinua ½ taza</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>atún 1½ lata(s), quinua 2 taza</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>atún 1½ lata(s), quinua 1½ taza</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>atún 1 lata(s), quinua 1 taza</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Cena: Frejoles guisados + ensalada + huevo</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>frejoles ¾ taza, huevo 1</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>frejoles 1 taza, huevo 1</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>frejoles 1½ taza, huevo 2</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>frejoles 1¼ taza, huevo 2</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>frejoles 1 taza, huevo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Almuerzo: Pescado a la plancha + papa + ensalada</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>pescado 150 g, papa 100 g</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>pescado 170 g, papa 100 g</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>pescado 250 g, papa 350 g</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>pescado 200 g, papa 250 g</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>pescado 150 g, papa 200 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Cena: Aguadito ligero de pollo</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>1 plato, pollo 100 g</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>1 plato, pollo 100 g</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>2 plato, pollo 150 g</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>1½ plato, pollo 120 g</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>1½ plato, pollo 100 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Almuerzo: Pollo salteado con brócoli + arroz integral</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>pollo 150 g, arroz ½ taza</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>pollo 170 g, arroz ½ taza</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>pollo 250 g, arroz 2 taza</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>pollo 200 g, arroz 1½ taza</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>pollo 150 g, arroz 1 taza</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Cena: Ensalada fría de lentejas + huevo</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>lentejas ¾ taza, huevo 1</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1 taza, huevo 1</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1½ taza, huevo 2</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1¼ taza, huevo 2</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>lentejas 1 taza, huevo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Almuerzo: Sudado de pescado + camote</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>pescado 150 g, camote 100 g</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>pescado 170 g, camote 100 g</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>pescado 250 g, camote 350 g</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>pescado 200 g, camote 250 g</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>pescado 150 g, camote 200 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Cena: Sopa de quinua con verduras + huevo</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>1 plato, huevo 1</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>1 plato, huevo 1</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>2 plato, huevo 2</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>1½ plato, huevo 2</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>1½ plato, huevo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr"/>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>DESAYUNOS</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Ella</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Él</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Hijo 18</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Hijo 16</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Hijo 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr"/>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Avena (días 1 y 4)</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>40 g avena, 200 ml leche descremada, 1 fruta chica, 1 huevo duro</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Igual que ella + 1 pan integral con ¼ palta</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>80 g avena, 300 ml leche, 1 plátano, 2 huevos, 2 panes integrales</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>60 g avena, 250 ml leche, 1 fruta, 2 huevos, 1 pan</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>50 g avena, 250 ml leche, 1 fruta, 1 huevo, 1 pan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr"/>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Pan integral con palta/queso + huevo (días 2 y 5)</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>1 pan, ¼ palta o 40 g queso, 1 huevo, 1 taza de papaya</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>2 panes, ¼ palta, 1 huevo, papaya</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>3 panes, ½ palta, 3 huevos, papaya, 250 ml leche</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>2–3 panes, ¼ palta o queso, 2 huevos, fruta</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>2 panes, 40 g queso, 1 huevo, fruta</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr"/>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Yogur con avena y fruta (días 3 y 6)</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>150 g yogur natural, 30 g avena, 1 fruta</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>200 g yogur, 40 g avena, 1 fruta, 1 huevo duro</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>300 g yogur, 60 g avena, 1 plátano, 1 cda mantequilla de maní, 2 huevos</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>250 g yogur, 50 g avena, 1 fruta, 1 pan</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>200 g yogur, 40 g avena, 1 fruta, 1 pan con queso</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr"/>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Huevos revueltos con pan (día 7)</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>2 huevos, 1 pan, fruta</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>2 huevos, 2 panes, fruta</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>4 huevos, 3 panes, fruta, 250 ml leche</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>3 huevos, 2 panes, fruta</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>2 huevos, 2 panes, fruta</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr"/>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>MEDIA TARDE</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Ella</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Él</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Hijo 18</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Hijo 16</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Hijo 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr"/>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Fruta + maní (días 1, 4 y 6)</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>1 fruta + 15 g maní</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>2 frutas + 15 g maní</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>2 frutas + 30 g maní + 1 pan con mantequilla de maní</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>1–2 frutas + 20 g maní + 1 pan</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>1 fruta + 15 g maní + yogur pequeño</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Yogur (días 2 y 5)</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>150 g yogur (+ plátano día 5)</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>200 g yogur + plátano</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>300 g yogur + plátano + 20 g maní</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>250 g yogur + plátano</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>200 g yogur + plátano</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr"/>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Fruta + queso fresco (días 3 y 7)</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>2 mandarinas o 1 naranja + 30 g queso</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>3 frutas + 30 g queso</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>3 frutas + 60 g queso + 1 pan</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>2 frutas + 40 g queso + 1 pan</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>2 frutas + 30 g queso</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Lunes a viernes</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
+        <is>
+          <t>Fin de semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Desayuno</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Recreo/lonchera (hijos 12 y 16)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Almuerzo</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>13:00 (hijos máx. 14:00)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Media tarde</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cena</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>19:00 (límite 19:30)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>19:30 (límite 20:00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cocina cerrada</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>21:00: solo agua o infusión</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>22:30–23:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar lista familiar con precios reales de Tottus y datos de etiquetas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pZgC66T2WsoYJHMycoAbf
</commit_message>
<xml_diff>
--- a/docs/seguimiento-dieta.xlsx
+++ b/docs/seguimiento-dieta.xlsx
@@ -2292,7 +2292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Atún en agua</t>
+          <t>Atún (filete en lata) [R]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>33</v>
+        <v>27.6</v>
       </c>
       <c r="E4" s="11" t="n"/>
       <c r="F4" s="5" t="n"/>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Huevos</t>
+          <t>Huevos, paquetes de 30 [R]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6 docenas</t>
+          <t>72 huevos (2,4 paquetes)</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>51</v>
+        <v>39.6</v>
       </c>
       <c r="E6" s="11" t="n"/>
       <c r="F6" s="5" t="n"/>
@@ -2479,16 +2479,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Queso fresco</t>
+          <t>Queso fresco [R]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>750 g</t>
+          <t>750 g (3 de 250 g)</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>19</v>
+        <v>50.7</v>
       </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="5" t="n"/>
@@ -2505,16 +2505,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yogur natural sin azúcar</t>
+          <t>Skyr natural 500 g, alta proteína [R]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3 kg</t>
+          <t>2 potes (1 kg)</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E8" s="11" t="n"/>
       <c r="F8" s="5" t="n"/>
@@ -2531,16 +2531,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Leche (UHT o fresca)</t>
+          <t>Yogur natural convencional</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>8 L</t>
+          <t>2 kg</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="E9" s="11" t="n"/>
       <c r="F9" s="5" t="n"/>
@@ -2552,21 +2552,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Menestras y granos</t>
+          <t>Proteínas y lácteos</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lentejas</t>
+          <t>Leche UHT entera [R]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1 kg</t>
+          <t>8 L</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>9</v>
+        <v>48.8</v>
       </c>
       <c r="E10" s="11" t="n"/>
       <c r="F10" s="5" t="n"/>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Frejoles</t>
+          <t>Lentejas [R]</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>12</v>
+        <v>7.2</v>
       </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="5" t="n"/>
@@ -2609,16 +2609,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Quinua</t>
+          <t>Frejoles [R]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>750 g</t>
+          <t>1 kg</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="5" t="n"/>
@@ -2635,16 +2635,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arroz integral</t>
+          <t>Quinua [R]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1,5 kg</t>
+          <t>750 g</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>15</v>
+        <v>10.4</v>
       </c>
       <c r="E13" s="11" t="n"/>
       <c r="F13" s="5" t="n"/>
@@ -2661,16 +2661,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Arroz blanco</t>
+          <t>Arroz integral</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2 kg</t>
+          <t>1,5 kg</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="5" t="n"/>
@@ -2687,16 +2687,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Avena en hojuelas</t>
+          <t>Arroz blanco</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1,2 kg</t>
+          <t>2 kg</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E15" s="11" t="n"/>
       <c r="F15" s="5" t="n"/>
@@ -2713,12 +2713,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pan integral</t>
+          <t>Avena en hojuelas 800 g [R]</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>3 bolsas</t>
+          <t>1,2 kg (1,5 bolsas)</t>
         </is>
       </c>
       <c r="D16" s="8" t="n">
@@ -2739,16 +2739,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fideos / pasta</t>
+          <t>Pan de quinua/integral [R]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1 kg</t>
+          <t>3 bolsas</t>
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>8</v>
+        <v>32.7</v>
       </c>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="5" t="n"/>
@@ -2760,21 +2760,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Verduras y tubérculos</t>
+          <t>Menestras y granos</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Camote</t>
+          <t>Fideos / spaghetti [R]</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3 kg</t>
+          <t>1 kg (2 de 500 g)</t>
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="5" t="n"/>
@@ -2791,16 +2791,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Papa</t>
+          <t>Camote [R]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4 kg</t>
+          <t>3 kg</t>
         </is>
       </c>
       <c r="D19" s="8" t="n">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="5" t="n"/>
@@ -2817,16 +2817,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Papa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3 kg</t>
+          <t>4 kg</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="5" t="n"/>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cebolla roja</t>
+          <t>Tomate [R]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>10.5</v>
+        <v>27.9</v>
       </c>
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="5" t="n"/>
@@ -2869,16 +2869,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Zanahoria</t>
+          <t>Cebolla roja</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2,5 kg</t>
+          <t>3 kg</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>7.5</v>
+        <v>10.5</v>
       </c>
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="5" t="n"/>
@@ -2895,16 +2895,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Espinaca</t>
+          <t>Zanahoria [R]</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>5 atados</t>
+          <t>2,5 kg</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="E23" s="11" t="n"/>
       <c r="F23" s="5" t="n"/>
@@ -2921,16 +2921,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Brócoli</t>
+          <t>Espinaca</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>3 unidades</t>
+          <t>5 atados</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="5" t="n"/>
@@ -2947,16 +2947,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Zapallo</t>
+          <t>Brócoli [R]</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1,5 kg</t>
+          <t>3 unidades</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>6</v>
+        <v>11.6</v>
       </c>
       <c r="E25" s="11" t="n"/>
       <c r="F25" s="5" t="n"/>
@@ -2973,16 +2973,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Choclo</t>
+          <t>Zapallo [R]</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4 unidades</t>
+          <t>1,5 kg</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="5" t="n"/>
@@ -2999,16 +2999,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Lechuga</t>
+          <t>Choclo [R]</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4 unidades</t>
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="5" t="n"/>
@@ -3025,16 +3025,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pepino</t>
+          <t>Lechuga [R]</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="5" t="n"/>
@@ -3051,16 +3051,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Arvejas</t>
+          <t>Pepino [R]</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>750 g</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>9</v>
+        <v>5.2</v>
       </c>
       <c r="E29" s="11" t="n"/>
       <c r="F29" s="5" t="n"/>
@@ -3077,16 +3077,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Limones</t>
+          <t>Arvejas [R]</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1,5 kg</t>
+          <t>750 g</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>12</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="5" t="n"/>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Palta</t>
+          <t>Limones [R]</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>8 unidades</t>
+          <t>1,5 kg</t>
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>24</v>
+        <v>5.6</v>
       </c>
       <c r="E31" s="11" t="n"/>
       <c r="F31" s="5" t="n"/>
@@ -3129,16 +3129,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ajo, culantro, perejil, ají amarillo</t>
+          <t>Palta fuerte [R]</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>varios</t>
+          <t>8 unidades</t>
         </is>
       </c>
       <c r="D32" s="8" t="n">
-        <v>15</v>
+        <v>41.7</v>
       </c>
       <c r="E32" s="11" t="n"/>
       <c r="F32" s="5" t="n"/>
@@ -3150,17 +3150,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Fruta</t>
+          <t>Verduras y tubérculos</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Plátano de seda</t>
+          <t>Ajo, culantro, perejil, ají amarillo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>≈30</t>
+          <t>varios</t>
         </is>
       </c>
       <c r="D33" s="8" t="n">
@@ -3181,16 +3181,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Manzana</t>
+          <t>Plátano de seda [R]</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>4 kg</t>
+          <t>≈30</t>
         </is>
       </c>
       <c r="D34" s="8" t="n">
-        <v>28</v>
+        <v>14.4</v>
       </c>
       <c r="E34" s="11" t="n"/>
       <c r="F34" s="5" t="n"/>
@@ -3207,16 +3207,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Papaya</t>
+          <t>Manzana Royal Gala [R]</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>3 medianas</t>
+          <t>4 kg</t>
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="E35" s="11" t="n"/>
       <c r="F35" s="5" t="n"/>
@@ -3233,16 +3233,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mandarina</t>
+          <t>Papaya [R]</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>3 kg</t>
+          <t>3 medianas</t>
         </is>
       </c>
       <c r="D36" s="8" t="n">
-        <v>13.5</v>
+        <v>30.7</v>
       </c>
       <c r="E36" s="11" t="n"/>
       <c r="F36" s="5" t="n"/>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Naranja</t>
+          <t>Mandarina</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3268,7 +3268,7 @@
         </is>
       </c>
       <c r="D37" s="8" t="n">
-        <v>10.5</v>
+        <v>13.5</v>
       </c>
       <c r="E37" s="11" t="n"/>
       <c r="F37" s="5" t="n"/>
@@ -3285,16 +3285,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Fruta de temporada (uvas, fresas, piña)</t>
+          <t>Naranja de jugo [R]</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2 kg</t>
+          <t>3 kg</t>
         </is>
       </c>
       <c r="D38" s="8" t="n">
-        <v>14</v>
+        <v>7.8</v>
       </c>
       <c r="E38" s="11" t="n"/>
       <c r="F38" s="5" t="n"/>
@@ -3306,21 +3306,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Grasas y frutos secos</t>
+          <t>Fruta</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Aceite de oliva extra virgen</t>
+          <t>Fruta de temporada (uva, piña) [R]</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>250 ml</t>
+          <t>2 kg</t>
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E39" s="11" t="n"/>
       <c r="F39" s="5" t="n"/>
@@ -3337,16 +3337,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Aceite vegetal</t>
+          <t>Aceite de oliva extra virgen</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1 L</t>
+          <t>250 ml</t>
         </is>
       </c>
       <c r="D40" s="8" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E40" s="11" t="n"/>
       <c r="F40" s="5" t="n"/>
@@ -3363,16 +3363,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Maní tostado sin sal</t>
+          <t>Aceite vegetal 900 ml [R]</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>600 g</t>
+          <t>1 botella</t>
         </is>
       </c>
       <c r="D41" s="8" t="n">
-        <v>20</v>
+        <v>5.7</v>
       </c>
       <c r="E41" s="11" t="n"/>
       <c r="F41" s="5" t="n"/>
@@ -3389,16 +3389,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mantequilla de maní natural</t>
+          <t>Maní tostado 250 g [R]</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1 frasco</t>
+          <t>750 g (3 potes)</t>
         </is>
       </c>
       <c r="D42" s="8" t="n">
-        <v>18</v>
+        <v>20.7</v>
       </c>
       <c r="E42" s="11" t="n"/>
       <c r="F42" s="5" t="n"/>
@@ -3410,21 +3410,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Despensa y antojos controlados</t>
+          <t>Grasas y frutos secos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Condimentos (sal, comino, orégano, ají panca)</t>
+          <t>Mantequilla de maní natural (La Purita, ~416 g) [R]</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>varios</t>
+          <t>1 frasco</t>
         </is>
       </c>
       <c r="D43" s="8" t="n">
-        <v>10</v>
+        <v>19.9</v>
       </c>
       <c r="E43" s="11" t="n"/>
       <c r="F43" s="5" t="n"/>
@@ -3441,16 +3441,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Azúcar</t>
+          <t>Condimentos (sal, comino, orégano, ají panca)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1 kg</t>
+          <t>varios</t>
         </is>
       </c>
       <c r="D44" s="8" t="n">
-        <v>4.5</v>
+        <v>10</v>
       </c>
       <c r="E44" s="11" t="n"/>
       <c r="F44" s="5" t="n"/>
@@ -3467,16 +3467,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Antojos: galletas integrales, chocolate amargo, canchita</t>
+          <t>Azúcar</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>presupuesto</t>
+          <t>1 kg</t>
         </is>
       </c>
       <c r="D45" s="8" t="n">
-        <v>25</v>
+        <v>4.5</v>
       </c>
       <c r="E45" s="11" t="n"/>
       <c r="F45" s="5" t="n"/>
@@ -3486,21 +3486,47 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="12" t="inlineStr">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Despensa y antojos controlados</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Antojos: galletas integrales, chocolate amargo, canchita</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>presupuesto</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="5" t="n"/>
+      <c r="G46" s="8">
+        <f>IF(E46="","",E46-D46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D46" s="8">
-        <f>SUM(D2:D45)</f>
-        <v/>
-      </c>
-      <c r="E46" s="8">
-        <f>SUM(E2:E45)</f>
-        <v/>
-      </c>
-      <c r="G46" s="8">
-        <f>IF(E46=0,"",E46-D46)</f>
+      <c r="D47" s="8">
+        <f>SUM(D2:D46)</f>
+        <v/>
+      </c>
+      <c r="E47" s="8">
+        <f>SUM(E2:E46)</f>
+        <v/>
+      </c>
+      <c r="G47" s="8">
+        <f>IF(E47=0,"",E47-D47)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar línea base de composición corporal y hoja de seguimiento
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pZgC66T2WsoYJHMycoAbf
</commit_message>
<xml_diff>
--- a/docs/seguimiento-dieta.xlsx
+++ b/docs/seguimiento-dieta.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras familia" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menú" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Porciones" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horarios" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composición" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compras familia" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menú" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Porciones" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horarios" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,6 +103,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1119,6 +1126,600 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Composición corporal (balanza de bioimpedancia). Medir siempre en las mismas condiciones: mañana, después de ir al baño, antes de comer/beber, sin ejercicio en las 12 h previas, pies limpios y secos. Valen las tendencias, no un solo dato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C3" s="18" t="inlineStr">
+        <is>
+          <t>ÉL peso (kg)</t>
+        </is>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>ÉL grasa (%)</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="inlineStr">
+        <is>
+          <t>ÉL grasa (kg)</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>ÉL masa magra (kg)</t>
+        </is>
+      </c>
+      <c r="G3" s="18" t="inlineStr">
+        <is>
+          <t>ÉL grasa visceral</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>ÉL agua (%)</t>
+        </is>
+      </c>
+      <c r="I3" s="18" t="inlineStr">
+        <is>
+          <t>ELLA peso (kg)</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
+        <is>
+          <t>ELLA grasa (%)</t>
+        </is>
+      </c>
+      <c r="K3" s="18" t="inlineStr">
+        <is>
+          <t>ELLA grasa (kg)</t>
+        </is>
+      </c>
+      <c r="L3" s="18" t="inlineStr">
+        <is>
+          <t>ELLA masa magra (kg)</t>
+        </is>
+      </c>
+      <c r="M3" s="18" t="inlineStr">
+        <is>
+          <t>ELLA grasa visceral</t>
+        </is>
+      </c>
+      <c r="N3" s="18" t="inlineStr">
+        <is>
+          <t>ELLA agua (%)</t>
+        </is>
+      </c>
+      <c r="O3" s="18" t="inlineStr">
+        <is>
+          <t>Δ grasa kg él / ella (vs sem. 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>línea base</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="E4" s="6">
+        <f>IF(AND(C4&lt;&gt;"",D4&lt;&gt;""),C4*D4/100,"")</f>
+        <v/>
+      </c>
+      <c r="F4" s="6">
+        <f>IF(E4&lt;&gt;"",C4-E4,"")</f>
+        <v/>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>89.25</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="K4" s="6">
+        <f>IF(AND(I4&lt;&gt;"",J4&lt;&gt;""),I4*J4/100,"")</f>
+        <v/>
+      </c>
+      <c r="L4" s="6">
+        <f>IF(K4&lt;&gt;"",I4-K4,"")</f>
+        <v/>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="O4">
+        <f>IF(AND(E4&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E4-$E$4,"0.0")&amp;" / "&amp;IF(K4&lt;&gt;"",TEXT(K4-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="6">
+        <f>IF(AND(C5&lt;&gt;"",D5&lt;&gt;""),C5*D5/100,"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="6">
+        <f>IF(E5&lt;&gt;"",C5-E5,"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="6">
+        <f>IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),I5*J5/100,"")</f>
+        <v/>
+      </c>
+      <c r="L5" s="6">
+        <f>IF(K5&lt;&gt;"",I5-K5,"")</f>
+        <v/>
+      </c>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5">
+        <f>IF(AND(E5&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E5-$E$4,"0.0")&amp;" / "&amp;IF(K5&lt;&gt;"",TEXT(K5-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6">
+        <f>IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),C6*D6/100,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="6">
+        <f>IF(E6&lt;&gt;"",C6-E6,"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="6">
+        <f>IF(AND(I6&lt;&gt;"",J6&lt;&gt;""),I6*J6/100,"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>IF(K6&lt;&gt;"",I6-K6,"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="5" t="n"/>
+      <c r="O6">
+        <f>IF(AND(E6&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E6-$E$4,"0.0")&amp;" / "&amp;IF(K6&lt;&gt;"",TEXT(K6-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="6">
+        <f>IF(AND(C7&lt;&gt;"",D7&lt;&gt;""),C7*D7/100,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="6">
+        <f>IF(E7&lt;&gt;"",C7-E7,"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="6">
+        <f>IF(AND(I7&lt;&gt;"",J7&lt;&gt;""),I7*J7/100,"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>IF(K7&lt;&gt;"",I7-K7,"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7">
+        <f>IF(AND(E7&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E7-$E$4,"0.0")&amp;" / "&amp;IF(K7&lt;&gt;"",TEXT(K7-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="6">
+        <f>IF(AND(C8&lt;&gt;"",D8&lt;&gt;""),C8*D8/100,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="6">
+        <f>IF(E8&lt;&gt;"",C8-E8,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="6">
+        <f>IF(AND(I8&lt;&gt;"",J8&lt;&gt;""),I8*J8/100,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>IF(K8&lt;&gt;"",I8-K8,"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="5" t="n"/>
+      <c r="O8">
+        <f>IF(AND(E8&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E8-$E$4,"0.0")&amp;" / "&amp;IF(K8&lt;&gt;"",TEXT(K8-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="6">
+        <f>IF(AND(C9&lt;&gt;"",D9&lt;&gt;""),C9*D9/100,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="6">
+        <f>IF(E9&lt;&gt;"",C9-E9,"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="6">
+        <f>IF(AND(I9&lt;&gt;"",J9&lt;&gt;""),I9*J9/100,"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>IF(K9&lt;&gt;"",I9-K9,"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="5" t="n"/>
+      <c r="O9">
+        <f>IF(AND(E9&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E9-$E$4,"0.0")&amp;" / "&amp;IF(K9&lt;&gt;"",TEXT(K9-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="6">
+        <f>IF(AND(C10&lt;&gt;"",D10&lt;&gt;""),C10*D10/100,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="6">
+        <f>IF(E10&lt;&gt;"",C10-E10,"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="6">
+        <f>IF(AND(I10&lt;&gt;"",J10&lt;&gt;""),I10*J10/100,"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="6">
+        <f>IF(K10&lt;&gt;"",I10-K10,"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="5" t="n"/>
+      <c r="O10">
+        <f>IF(AND(E10&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E10-$E$4,"0.0")&amp;" / "&amp;IF(K10&lt;&gt;"",TEXT(K10-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="6">
+        <f>IF(AND(C11&lt;&gt;"",D11&lt;&gt;""),C11*D11/100,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="6">
+        <f>IF(E11&lt;&gt;"",C11-E11,"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="6">
+        <f>IF(AND(I11&lt;&gt;"",J11&lt;&gt;""),I11*J11/100,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>IF(K11&lt;&gt;"",I11-K11,"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="5" t="n"/>
+      <c r="O11">
+        <f>IF(AND(E11&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E11-$E$4,"0.0")&amp;" / "&amp;IF(K11&lt;&gt;"",TEXT(K11-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="6">
+        <f>IF(AND(C12&lt;&gt;"",D12&lt;&gt;""),C12*D12/100,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="6">
+        <f>IF(E12&lt;&gt;"",C12-E12,"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="6">
+        <f>IF(AND(I12&lt;&gt;"",J12&lt;&gt;""),I12*J12/100,"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>IF(K12&lt;&gt;"",I12-K12,"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="5" t="n"/>
+      <c r="O12">
+        <f>IF(AND(E12&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E12-$E$4,"0.0")&amp;" / "&amp;IF(K12&lt;&gt;"",TEXT(K12-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="6">
+        <f>IF(AND(C13&lt;&gt;"",D13&lt;&gt;""),C13*D13/100,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="6">
+        <f>IF(E13&lt;&gt;"",C13-E13,"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="6">
+        <f>IF(AND(I13&lt;&gt;"",J13&lt;&gt;""),I13*J13/100,"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>IF(K13&lt;&gt;"",I13-K13,"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="5" t="n"/>
+      <c r="O13">
+        <f>IF(AND(E13&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E13-$E$4,"0.0")&amp;" / "&amp;IF(K13&lt;&gt;"",TEXT(K13-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="6">
+        <f>IF(AND(C14&lt;&gt;"",D14&lt;&gt;""),C14*D14/100,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="6">
+        <f>IF(E14&lt;&gt;"",C14-E14,"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="6">
+        <f>IF(AND(I14&lt;&gt;"",J14&lt;&gt;""),I14*J14/100,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>IF(K14&lt;&gt;"",I14-K14,"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
+      <c r="O14">
+        <f>IF(AND(E14&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E14-$E$4,"0.0")&amp;" / "&amp;IF(K14&lt;&gt;"",TEXT(K14-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="6">
+        <f>IF(AND(C15&lt;&gt;"",D15&lt;&gt;""),C15*D15/100,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>IF(E15&lt;&gt;"",C15-E15,"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="6">
+        <f>IF(AND(I15&lt;&gt;"",J15&lt;&gt;""),I15*J15/100,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>IF(K15&lt;&gt;"",I15-K15,"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+      <c r="O15">
+        <f>IF(AND(E15&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E15-$E$4,"0.0")&amp;" / "&amp;IF(K15&lt;&gt;"",TEXT(K15-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="6">
+        <f>IF(AND(C16&lt;&gt;"",D16&lt;&gt;""),C16*D16/100,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>IF(E16&lt;&gt;"",C16-E16,"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="6">
+        <f>IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),I16*J16/100,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>IF(K16&lt;&gt;"",I16-K16,"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="5" t="n"/>
+      <c r="O16">
+        <f>IF(AND(E16&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E16-$E$4,"0.0")&amp;" / "&amp;IF(K16&lt;&gt;"",TEXT(K16-$K$4,"0.0"),"-"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Línea base (semana 0) tomada de la balanza: Él 78,6 kg, 27,7 % grasa, visceral 12; Ella 89,25 kg, 51,8 % grasa, visceral 14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Las metas que sugiere la app de la balanza ("peso estándar", -11,8 kg y -33,3 kg) son genéricas; usar metas por etapas (5-10 % del peso) y validarlas con el médico.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1164,10 +1765,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>76</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>86</v>
+        <v>89.25</v>
       </c>
     </row>
     <row r="4">
@@ -1316,7 +1917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2286,7 +2887,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3535,7 +4136,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3765,7 +4366,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4630,7 +5231,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Registrar talla, cintura y brazo en la línea base
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pZgC66T2WsoYJHMycoAbf
</commit_message>
<xml_diff>
--- a/docs/seguimiento-dieta.xlsx
+++ b/docs/seguimiento-dieta.xlsx
@@ -605,8 +605,12 @@
         <f>Perfil!C3</f>
         <v/>
       </c>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
+      <c r="E5" s="5" t="n">
+        <v>103</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>105</v>
+      </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="5" t="n"/>
@@ -1126,7 +1130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1144,6 +1148,8 @@
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
@@ -1229,6 +1235,16 @@
           <t>Δ grasa kg él / ella (vs sem. 0)</t>
         </is>
       </c>
+      <c r="P3" s="18" t="inlineStr">
+        <is>
+          <t>ÉL brazo (cm)</t>
+        </is>
+      </c>
+      <c r="Q3" s="18" t="inlineStr">
+        <is>
+          <t>ELLA brazo (cm)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1282,6 +1298,12 @@
       <c r="O4">
         <f>IF(AND(E4&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E4-$E$4,"0.0")&amp;" / "&amp;IF(K4&lt;&gt;"",TEXT(K4-$K$4,"0.0"),"-"),"")</f>
         <v/>
+      </c>
+      <c r="P4" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -1317,6 +1339,8 @@
         <f>IF(AND(E5&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E5-$E$4,"0.0")&amp;" / "&amp;IF(K5&lt;&gt;"",TEXT(K5-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1351,6 +1375,8 @@
         <f>IF(AND(E6&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E6-$E$4,"0.0")&amp;" / "&amp;IF(K6&lt;&gt;"",TEXT(K6-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1385,6 +1411,8 @@
         <f>IF(AND(E7&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E7-$E$4,"0.0")&amp;" / "&amp;IF(K7&lt;&gt;"",TEXT(K7-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1419,6 +1447,8 @@
         <f>IF(AND(E8&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E8-$E$4,"0.0")&amp;" / "&amp;IF(K8&lt;&gt;"",TEXT(K8-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1453,6 +1483,8 @@
         <f>IF(AND(E9&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E9-$E$4,"0.0")&amp;" / "&amp;IF(K9&lt;&gt;"",TEXT(K9-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P9" s="5" t="n"/>
+      <c r="Q9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1487,6 +1519,8 @@
         <f>IF(AND(E10&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E10-$E$4,"0.0")&amp;" / "&amp;IF(K10&lt;&gt;"",TEXT(K10-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1521,6 +1555,8 @@
         <f>IF(AND(E11&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E11-$E$4,"0.0")&amp;" / "&amp;IF(K11&lt;&gt;"",TEXT(K11-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P11" s="5" t="n"/>
+      <c r="Q11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1555,6 +1591,8 @@
         <f>IF(AND(E12&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E12-$E$4,"0.0")&amp;" / "&amp;IF(K12&lt;&gt;"",TEXT(K12-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1589,6 +1627,8 @@
         <f>IF(AND(E13&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E13-$E$4,"0.0")&amp;" / "&amp;IF(K13&lt;&gt;"",TEXT(K13-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P13" s="5" t="n"/>
+      <c r="Q13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1623,6 +1663,8 @@
         <f>IF(AND(E14&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E14-$E$4,"0.0")&amp;" / "&amp;IF(K14&lt;&gt;"",TEXT(K14-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1657,6 +1699,8 @@
         <f>IF(AND(E15&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E15-$E$4,"0.0")&amp;" / "&amp;IF(K15&lt;&gt;"",TEXT(K15-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P15" s="5" t="n"/>
+      <c r="Q15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1691,6 +1735,8 @@
         <f>IF(AND(E16&lt;&gt;"",$E$4&lt;&gt;""),TEXT(E16-$E$4,"0.0")&amp;" / "&amp;IF(K16&lt;&gt;"",TEXT(K16-$K$4,"0.0"),"-"),"")</f>
         <v/>
       </c>
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1703,6 +1749,13 @@
       <c r="A19" t="inlineStr">
         <is>
           <t>Las metas que sugiere la app de la balanza ("peso estándar", -11,8 kg y -33,3 kg) son genéricas; usar metas por etapas (5-10 % del peso) y validarlas con el médico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Brazo: medir relajado, a la mitad entre hombro y codo. Cintura: a la altura del ombligo, al final de una exhalación normal.</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1778,7 +1831,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>150</v>
@@ -1910,6 +1963,21 @@
         <is>
           <t>Nota: para ella la proteína por peso real da un valor alto; usar ~80-95 g (peso ajustado) salvo indicación médica.</t>
         </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Relación cintura/talla (&lt; 0,5 deseable)</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>Seguimiento!E5/B4</f>
+        <v/>
+      </c>
+      <c r="C18" s="8">
+        <f>Seguimiento!F5/C4</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>